<commit_message>
Make the current-state spreadsheet slide show unexplained variance.
</commit_message>
<xml_diff>
--- a/deck/Northline_HC_Recon_FICTIONAL.xlsx
+++ b/deck/Northline_HC_Recon_FICTIONAL.xlsx
@@ -22,17 +22,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -43,21 +39,13 @@
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -72,14 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,50 +430,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="B1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Latest Department</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Latest Org</t>
         </is>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="F1" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="H1" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="I1" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="1" t="n">
         <v>46296</v>
       </c>
-      <c r="K1" s="2" t="n">
+      <c r="K1" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="L1" s="2" t="n">
+      <c r="L1" s="1" t="n">
         <v>46357</v>
       </c>
     </row>
@@ -509,25 +493,25 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -547,25 +531,25 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -585,25 +569,25 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -623,25 +607,25 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -661,25 +645,25 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -699,25 +683,25 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -737,25 +721,25 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -851,25 +835,25 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -889,25 +873,25 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -965,25 +949,25 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1003,25 +987,25 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1079,25 +1063,25 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="J17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
@@ -1117,25 +1101,25 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="J18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="K18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="L18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -1155,25 +1139,25 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20">
@@ -1193,25 +1177,25 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1231,25 +1215,25 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1269,25 +1253,25 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -1307,25 +1291,25 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -1345,25 +1329,25 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1383,25 +1367,25 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1421,25 +1405,25 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1497,25 +1481,25 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1535,25 +1519,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
@@ -1573,25 +1557,25 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1611,25 +1595,25 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1649,25 +1633,25 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -1687,25 +1671,25 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1725,25 +1709,25 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -1763,25 +1747,25 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="I35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="J35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="K35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="L35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -1801,25 +1785,25 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -1839,25 +1823,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -1877,25 +1861,25 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="K38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39">
@@ -1915,25 +1899,25 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -1991,25 +1975,25 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="L41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42">
@@ -2029,25 +2013,25 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -2067,25 +2051,25 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -2105,25 +2089,25 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2137,50 +2121,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="B1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Latest Department</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Latest Org</t>
         </is>
       </c>
-      <c r="F1" s="2" t="n">
+      <c r="F1" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="G1" s="2" t="n">
+      <c r="G1" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="H1" s="2" t="n">
+      <c r="H1" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="I1" s="2" t="n">
+      <c r="I1" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="J1" s="2" t="n">
+      <c r="J1" s="1" t="n">
         <v>46296</v>
       </c>
-      <c r="K1" s="2" t="n">
+      <c r="K1" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="L1" s="2" t="n">
+      <c r="L1" s="1" t="n">
         <v>46357</v>
       </c>
     </row>
@@ -2201,25 +2179,25 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -2239,25 +2217,25 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -2277,25 +2255,25 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2315,25 +2293,25 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -2353,25 +2331,25 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -2391,25 +2369,25 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -2429,25 +2407,25 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -2508,22 +2486,22 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2543,25 +2521,25 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2581,25 +2559,25 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2625,7 +2603,7 @@
         <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
@@ -2657,25 +2635,25 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2695,25 +2673,25 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2742,16 +2720,16 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2771,25 +2749,25 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="H17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="I17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="J17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="K17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="L17" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -2809,25 +2787,25 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="H18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="I18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="K18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="L18" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -2847,25 +2825,25 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20">
@@ -2885,25 +2863,25 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -2923,25 +2901,25 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2961,25 +2939,25 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -2999,13 +2977,13 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
         <v>2</v>
@@ -3037,25 +3015,25 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -3075,25 +3053,25 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -3113,25 +3091,25 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -3189,25 +3167,25 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -3227,25 +3205,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30">
@@ -3265,25 +3243,25 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -3303,25 +3281,25 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3341,25 +3319,25 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33">
@@ -3379,25 +3357,25 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -3417,25 +3395,25 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -3455,25 +3433,25 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="H35" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="I35" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="J35" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="K35" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="L35" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36">
@@ -3493,25 +3471,25 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -3531,25 +3509,25 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -3569,25 +3547,25 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="K38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39">
@@ -3607,25 +3585,25 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="I39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -3683,25 +3661,25 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="L41" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42">
@@ -3721,25 +3699,25 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -3759,25 +3737,25 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -3797,25 +3775,25 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3829,48 +3807,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Headcount Reconciliation — Approved Plan (as of 6/30/26) vs. Working Plan / Roll Forward (as of 7/31/26)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Northline Systems — FICTIONAL DEMO DATA (structure inspired by a real multi-tab recon workbook)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Total Headcount</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="1" t="n">
         <v>46296</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="N4" s="1" t="n">
         <v>46357</v>
       </c>
     </row>
@@ -3881,25 +3854,25 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="I5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="J5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="K5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="L5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="M5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="N5" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6">
@@ -3909,25 +3882,25 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>277</v>
+        <v>251</v>
       </c>
       <c r="I6" t="n">
-        <v>277</v>
+        <v>246</v>
       </c>
       <c r="J6" t="n">
-        <v>273</v>
+        <v>246</v>
       </c>
       <c r="K6" t="n">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="L6" t="n">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="M6" t="n">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="N6" t="n">
-        <v>274</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7">
@@ -3940,1732 +3913,22 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="J7" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="K7" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="L7" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="M7" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="N7" t="n">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Roster — All Roles by Org and Department</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Role Detail</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Approved Plan (presented 6/30)</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Working Plan (as of 7/31)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Org</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Jul</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Aug</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Jun</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Jul</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Aug</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Δ Jul</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Director of Partnerships</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>12</v>
-      </c>
-      <c r="I13" t="n">
-        <v>12</v>
-      </c>
-      <c r="J13" t="n">
-        <v>12</v>
-      </c>
-      <c r="O13" t="n">
-        <v>12</v>
-      </c>
-      <c r="P13" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>11</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Partner Success Manager</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>VP Sales</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>1</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Account Executive</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>1</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Outbound AE</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>12</v>
-      </c>
-      <c r="I17" t="n">
-        <v>12</v>
-      </c>
-      <c r="J17" t="n">
-        <v>12</v>
-      </c>
-      <c r="O17" t="n">
-        <v>12</v>
-      </c>
-      <c r="P17" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>12</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>SDR</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Demand Gen Manager</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>3</v>
-      </c>
-      <c r="I19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" t="n">
-        <v>3</v>
-      </c>
-      <c r="O19" t="n">
-        <v>3</v>
-      </c>
-      <c r="P19" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>3</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Content Manager</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Events Marketing Manager</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>1</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Lifecycle Marketing Manager</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" t="n">
-        <v>6</v>
-      </c>
-      <c r="J22" t="n">
-        <v>6</v>
-      </c>
-      <c r="O22" t="n">
-        <v>6</v>
-      </c>
-      <c r="P22" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>6</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Product Marketing Manager</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Staff Platform Engineer</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>1</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Sr. Backend Engineer</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" t="n">
-        <v>3</v>
-      </c>
-      <c r="J25" t="n">
-        <v>3</v>
-      </c>
-      <c r="O25" t="n">
-        <v>3</v>
-      </c>
-      <c r="P25" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>3</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>4</v>
-      </c>
-      <c r="I26" t="n">
-        <v>4</v>
-      </c>
-      <c r="J26" t="n">
-        <v>4</v>
-      </c>
-      <c r="O26" t="n">
-        <v>4</v>
-      </c>
-      <c r="P26" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>4</v>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>QA Manager</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" t="n">
-        <v>1</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" t="n">
-        <v>1</v>
-      </c>
-      <c r="P27" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>1</v>
-      </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H28" t="n">
-        <v>24</v>
-      </c>
-      <c r="I28" t="n">
-        <v>24</v>
-      </c>
-      <c r="J28" t="n">
-        <v>24</v>
-      </c>
-      <c r="O28" t="n">
-        <v>24</v>
-      </c>
-      <c r="P28" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>24</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Product Manager — Growth</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>18</v>
-      </c>
-      <c r="I29" t="n">
-        <v>18</v>
-      </c>
-      <c r="J29" t="n">
-        <v>18</v>
-      </c>
-      <c r="O29" t="n">
-        <v>18</v>
-      </c>
-      <c r="P29" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>18</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Product Analyst</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>2</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2</v>
-      </c>
-      <c r="J30" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" t="n">
-        <v>2</v>
-      </c>
-      <c r="P30" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>2</v>
-      </c>
-      <c r="R30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Head of Product</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H31" t="n">
-        <v>1</v>
-      </c>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" t="n">
-        <v>1</v>
-      </c>
-      <c r="P31" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>1</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Product Designer</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>24</v>
-      </c>
-      <c r="I32" t="n">
-        <v>24</v>
-      </c>
-      <c r="J32" t="n">
-        <v>24</v>
-      </c>
-      <c r="O32" t="n">
-        <v>24</v>
-      </c>
-      <c r="P32" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>24</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Senior Product Designer</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Technical Success Manager</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Customer Success</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>3</v>
-      </c>
-      <c r="I34" t="n">
-        <v>3</v>
-      </c>
-      <c r="J34" t="n">
-        <v>3</v>
-      </c>
-      <c r="O34" t="n">
-        <v>3</v>
-      </c>
-      <c r="P34" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>3</v>
-      </c>
-      <c r="R34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Customer Success Manager</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Customer Success</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2</v>
-      </c>
-      <c r="J35" t="n">
-        <v>2</v>
-      </c>
-      <c r="O35" t="n">
-        <v>2</v>
-      </c>
-      <c r="P35" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>1</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Technical Account Manager</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Customer Success</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>8</v>
-      </c>
-      <c r="I36" t="n">
-        <v>8</v>
-      </c>
-      <c r="J36" t="n">
-        <v>8</v>
-      </c>
-      <c r="O36" t="n">
-        <v>8</v>
-      </c>
-      <c r="P36" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>8</v>
-      </c>
-      <c r="R36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>FP&amp;A Analyst</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>24</v>
-      </c>
-      <c r="I37" t="n">
-        <v>24</v>
-      </c>
-      <c r="J37" t="n">
-        <v>24</v>
-      </c>
-      <c r="O37" t="n">
-        <v>24</v>
-      </c>
-      <c r="P37" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>24</v>
-      </c>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Controller</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H38" t="n">
-        <v>18</v>
-      </c>
-      <c r="I38" t="n">
-        <v>18</v>
-      </c>
-      <c r="J38" t="n">
-        <v>18</v>
-      </c>
-      <c r="O38" t="n">
-        <v>18</v>
-      </c>
-      <c r="P38" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>18</v>
-      </c>
-      <c r="R38" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>HRBP</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>6</v>
-      </c>
-      <c r="I39" t="n">
-        <v>6</v>
-      </c>
-      <c r="J39" t="n">
-        <v>6</v>
-      </c>
-      <c r="O39" t="n">
-        <v>6</v>
-      </c>
-      <c r="P39" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>6</v>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Recruiter</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H40" t="n">
-        <v>3</v>
-      </c>
-      <c r="I40" t="n">
-        <v>3</v>
-      </c>
-      <c r="J40" t="n">
-        <v>3</v>
-      </c>
-      <c r="O40" t="n">
-        <v>3</v>
-      </c>
-      <c r="P40" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>3</v>
-      </c>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Office Manager</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>6</v>
-      </c>
-      <c r="I41" t="n">
-        <v>6</v>
-      </c>
-      <c r="J41" t="n">
-        <v>6</v>
-      </c>
-      <c r="O41" t="n">
-        <v>6</v>
-      </c>
-      <c r="P41" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>6</v>
-      </c>
-      <c r="R41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>IT Support</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>12</v>
-      </c>
-      <c r="I42" t="n">
-        <v>12</v>
-      </c>
-      <c r="J42" t="n">
-        <v>12</v>
-      </c>
-      <c r="O42" t="n">
-        <v>12</v>
-      </c>
-      <c r="P42" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>12</v>
-      </c>
-      <c r="R42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Software Engineer II</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>2</v>
-      </c>
-      <c r="I43" t="n">
-        <v>2</v>
-      </c>
-      <c r="J43" t="n">
-        <v>2</v>
-      </c>
-      <c r="O43" t="n">
-        <v>2</v>
-      </c>
-      <c r="P43" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>2</v>
-      </c>
-      <c r="R43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Software Engineer I</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H44" t="n">
-        <v>1</v>
-      </c>
-      <c r="I44" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" t="n">
-        <v>1</v>
-      </c>
-      <c r="O44" t="n">
-        <v>1</v>
-      </c>
-      <c r="P44" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>1</v>
-      </c>
-      <c r="R44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Principal Engineer</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>0</v>
-      </c>
-      <c r="R45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Sales Manager</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H46" t="n">
-        <v>24</v>
-      </c>
-      <c r="I46" t="n">
-        <v>24</v>
-      </c>
-      <c r="J46" t="n">
-        <v>24</v>
-      </c>
-      <c r="O46" t="n">
-        <v>24</v>
-      </c>
-      <c r="P46" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>23</v>
-      </c>
-      <c r="R46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Enterprise BDR</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>0</v>
-      </c>
-      <c r="R47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Brand Manager</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Marketing Ops</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H49" t="n">
-        <v>1</v>
-      </c>
-      <c r="I49" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" t="n">
-        <v>1</v>
-      </c>
-      <c r="O49" t="n">
-        <v>1</v>
-      </c>
-      <c r="P49" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>1</v>
-      </c>
-      <c r="R49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Design Manager</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H50" t="n">
-        <v>12</v>
-      </c>
-      <c r="I50" t="n">
-        <v>12</v>
-      </c>
-      <c r="J50" t="n">
-        <v>12</v>
-      </c>
-      <c r="O50" t="n">
-        <v>12</v>
-      </c>
-      <c r="P50" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>12</v>
-      </c>
-      <c r="R50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Content Designer</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>1</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" t="n">
-        <v>1</v>
-      </c>
-      <c r="O51" t="n">
-        <v>1</v>
-      </c>
-      <c r="P51" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>1</v>
-      </c>
-      <c r="R51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>CS Director</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Customer Success</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>2</v>
-      </c>
-      <c r="I52" t="n">
-        <v>2</v>
-      </c>
-      <c r="J52" t="n">
-        <v>2</v>
-      </c>
-      <c r="O52" t="n">
-        <v>2</v>
-      </c>
-      <c r="P52" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>2</v>
-      </c>
-      <c r="R52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Staff Accountant</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>12</v>
-      </c>
-      <c r="I53" t="n">
-        <v>12</v>
-      </c>
-      <c r="J53" t="n">
-        <v>12</v>
-      </c>
-      <c r="O53" t="n">
-        <v>12</v>
-      </c>
-      <c r="P53" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>12</v>
-      </c>
-      <c r="R53" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>HR Generalist</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>18</v>
-      </c>
-      <c r="I54" t="n">
-        <v>18</v>
-      </c>
-      <c r="J54" t="n">
-        <v>18</v>
-      </c>
-      <c r="O54" t="n">
-        <v>18</v>
-      </c>
-      <c r="P54" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>18</v>
-      </c>
-      <c r="R54" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>People Ops Manager</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>G&amp;A</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>8</v>
-      </c>
-      <c r="I55" t="n">
-        <v>8</v>
-      </c>
-      <c r="J55" t="n">
-        <v>8</v>
-      </c>
-      <c r="O55" t="n">
-        <v>8</v>
-      </c>
-      <c r="P55" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>8</v>
-      </c>
-      <c r="R55" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
     </row>
   </sheetData>
@@ -5679,7 +3942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5689,265 +3952,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Each row is a month-over-month headcount increase in the roll-forward tab. Fictional demo data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>RF Row</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Org</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Net Adds</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Rec Needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>16</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Outbound AE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Above-plan request — pending finance</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" t="n">
-        <v>12</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Staff Platform Engineer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Approved plan net-new</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" t="n">
-        <v>17</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Product Analyst</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Start slipped from Aug</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" t="n">
-        <v>19</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Product Designer</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" t="n">
-        <v>9</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Events Marketing Manager</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>GTM</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Not backfilling — explained variance</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>